<commit_message>
feat: auto-append forecast to 广东日前电价预测.xlsx
</commit_message>
<xml_diff>
--- a/广东日前电价预测.xlsx
+++ b/广东日前电价预测.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="31120" windowHeight="13760"/>
+    <workbookView windowWidth="31120" windowHeight="13700"/>
   </bookViews>
   <sheets>
     <sheet name="电价预测" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>日期</t>
   </si>
@@ -123,6 +123,9 @@
   </si>
   <si>
     <t>2026-06-04</t>
+  </si>
+  <si>
+    <t>2026-06-05</t>
   </si>
 </sst>
 </file>
@@ -1121,7 +1124,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Z9"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1693,163 +1696,323 @@
       </c>
     </row>
     <row r="8" spans="1:26">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="4">
         <v>477.510083312321</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <v>460.179972585153</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="4">
         <v>452.272309581806</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="4">
         <v>446.698428702462</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="4">
         <v>435.203170943753</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="4">
         <v>423.167495978268</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="4">
         <v>416.665204093686</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="4">
         <v>405.594452801676</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="4">
         <v>410.657806080651</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="4">
         <v>408.64571872195</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="4">
         <v>392.786665586946</v>
       </c>
-      <c r="N8" s="5">
+      <c r="N8" s="4">
         <v>397.551514717864</v>
       </c>
-      <c r="O8" s="5">
+      <c r="O8" s="4">
         <v>377.287011715518</v>
       </c>
-      <c r="P8" s="5">
+      <c r="P8" s="4">
         <v>439.802507228529</v>
       </c>
-      <c r="Q8" s="5">
+      <c r="Q8" s="4">
         <v>419.579326094659</v>
       </c>
-      <c r="R8" s="5">
+      <c r="R8" s="4">
         <v>427.253618776202</v>
       </c>
-      <c r="S8" s="5">
+      <c r="S8" s="4">
         <v>473.537313440555</v>
       </c>
-      <c r="T8" s="5">
+      <c r="T8" s="4">
         <v>504.83846731029</v>
       </c>
-      <c r="U8" s="5">
+      <c r="U8" s="4">
         <v>538.040234576353</v>
       </c>
-      <c r="V8" s="5">
+      <c r="V8" s="4">
         <v>584.680684992047</v>
       </c>
-      <c r="W8" s="5">
+      <c r="W8" s="4">
         <v>558.410842207158</v>
       </c>
-      <c r="X8" s="5">
+      <c r="X8" s="4">
         <v>560.718673726151</v>
       </c>
-      <c r="Y8" s="5">
+      <c r="Y8" s="4">
         <v>553.059204414606</v>
       </c>
-      <c r="Z8" s="5">
+      <c r="Z8" s="4">
         <v>532.850782162577</v>
       </c>
     </row>
     <row r="9" spans="1:26">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="4">
         <v>479.663105278797</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="4">
         <v>450.226060237573</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="4">
         <v>446.49602201333</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="4">
         <v>441.516101643513</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <v>436.723535932768</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="4">
         <v>426.273717778106</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="4">
         <v>415.471833490793</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="4">
         <v>405.395435743732</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="4">
         <v>405.526210693069</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="4">
         <v>401.24318723317</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="4">
         <v>395.367585233927</v>
       </c>
-      <c r="N9" s="5">
+      <c r="N9" s="4">
         <v>400.419861508885</v>
       </c>
-      <c r="O9" s="5">
+      <c r="O9" s="4">
         <v>374.85397893975</v>
       </c>
-      <c r="P9" s="5">
+      <c r="P9" s="4">
         <v>430.488614133024</v>
       </c>
-      <c r="Q9" s="5">
+      <c r="Q9" s="4">
         <v>415.335700830734</v>
       </c>
-      <c r="R9" s="5">
+      <c r="R9" s="4">
         <v>422.568728061064</v>
       </c>
-      <c r="S9" s="5">
+      <c r="S9" s="4">
         <v>461.639028421042</v>
       </c>
-      <c r="T9" s="5">
+      <c r="T9" s="4">
         <v>474.159354650376</v>
       </c>
-      <c r="U9" s="5">
+      <c r="U9" s="4">
         <v>559.281670901527</v>
       </c>
-      <c r="V9" s="5">
+      <c r="V9" s="4">
         <v>585.692266672926</v>
       </c>
-      <c r="W9" s="5">
+      <c r="W9" s="4">
         <v>571.248928756925</v>
       </c>
-      <c r="X9" s="5">
+      <c r="X9" s="4">
         <v>570.213680505303</v>
       </c>
-      <c r="Y9" s="5">
+      <c r="Y9" s="4">
         <v>564.381001825957</v>
       </c>
-      <c r="Z9" s="5">
+      <c r="Z9" s="4">
         <v>541.969986591737</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26">
+      <c r="A10" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="5">
+        <v>499.999953314644</v>
+      </c>
+      <c r="D10" s="5">
+        <v>453.072393128946</v>
+      </c>
+      <c r="E10" s="5">
+        <v>439.191376099889</v>
+      </c>
+      <c r="F10" s="5">
+        <v>432.016780667161</v>
+      </c>
+      <c r="G10" s="5">
+        <v>407.277749180335</v>
+      </c>
+      <c r="H10" s="5">
+        <v>416.156810739828</v>
+      </c>
+      <c r="I10" s="5">
+        <v>396.460923928478</v>
+      </c>
+      <c r="J10" s="5">
+        <v>385.469848189552</v>
+      </c>
+      <c r="K10" s="5">
+        <v>406.417160490052</v>
+      </c>
+      <c r="L10" s="5">
+        <v>410.327960088287</v>
+      </c>
+      <c r="M10" s="5">
+        <v>395.842158654537</v>
+      </c>
+      <c r="N10" s="5">
+        <v>404.988435928563</v>
+      </c>
+      <c r="O10" s="5">
+        <v>395.61937094767</v>
+      </c>
+      <c r="P10" s="5">
+        <v>449.579844359478</v>
+      </c>
+      <c r="Q10" s="5">
+        <v>427.220788940556</v>
+      </c>
+      <c r="R10" s="5">
+        <v>449.693058150572</v>
+      </c>
+      <c r="S10" s="5">
+        <v>482.716871633252</v>
+      </c>
+      <c r="T10" s="5">
+        <v>503.372417895902</v>
+      </c>
+      <c r="U10" s="5">
+        <v>543.090929658904</v>
+      </c>
+      <c r="V10" s="5">
+        <v>584.52033161696</v>
+      </c>
+      <c r="W10" s="5">
+        <v>553.942760700385</v>
+      </c>
+      <c r="X10" s="5">
+        <v>566.9670145727</v>
+      </c>
+      <c r="Y10" s="5">
+        <v>562.773969342367</v>
+      </c>
+      <c r="Z10" s="5">
+        <v>504.491941381037</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26">
+      <c r="A11" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="5">
+        <v>491.633524173506</v>
+      </c>
+      <c r="D11" s="5">
+        <v>453.101802437633</v>
+      </c>
+      <c r="E11" s="5">
+        <v>446.34160846947</v>
+      </c>
+      <c r="F11" s="5">
+        <v>439.628730505544</v>
+      </c>
+      <c r="G11" s="5">
+        <v>424.74350339526</v>
+      </c>
+      <c r="H11" s="5">
+        <v>421.494928893309</v>
+      </c>
+      <c r="I11" s="5">
+        <v>403.497951718332</v>
+      </c>
+      <c r="J11" s="5">
+        <v>394.583568771318</v>
+      </c>
+      <c r="K11" s="5">
+        <v>404.804859829541</v>
+      </c>
+      <c r="L11" s="5">
+        <v>409.195955870284</v>
+      </c>
+      <c r="M11" s="5">
+        <v>400.631554406933</v>
+      </c>
+      <c r="N11" s="5">
+        <v>407.249978603199</v>
+      </c>
+      <c r="O11" s="5">
+        <v>394.546730712444</v>
+      </c>
+      <c r="P11" s="5">
+        <v>441.223942478279</v>
+      </c>
+      <c r="Q11" s="5">
+        <v>424.31534979812</v>
+      </c>
+      <c r="R11" s="5">
+        <v>439.642650357999</v>
+      </c>
+      <c r="S11" s="5">
+        <v>460.236281488575</v>
+      </c>
+      <c r="T11" s="5">
+        <v>472.289916725599</v>
+      </c>
+      <c r="U11" s="5">
+        <v>543.462612053415</v>
+      </c>
+      <c r="V11" s="5">
+        <v>560.216553982182</v>
+      </c>
+      <c r="W11" s="5">
+        <v>540.307229292708</v>
+      </c>
+      <c r="X11" s="5">
+        <v>538.756485421846</v>
+      </c>
+      <c r="Y11" s="5">
+        <v>541.227909112238</v>
+      </c>
+      <c r="Z11" s="5">
+        <v>514.952669537084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>